<commit_message>
refactor(docs): examples engine playground & landing
</commit_message>
<xml_diff>
--- a/apps/docs/public/generated/examples/showcase/native-excel-forecast-table/artifact/native-excel-forecast-table.xlsx
+++ b/apps/docs/public/generated/examples/showcase/native-excel-forecast-table/artifact/native-excel-forecast-table.xlsx
@@ -126,16 +126,20 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF1E3A8A"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -147,12 +151,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE9E9E9"/>
+        <fgColor rgb="FFDBEAFE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9E9E9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -214,16 +224,16 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>